<commit_message>
feat: importacao opcional de marca/fabricante/part_number e selecao multipla de produtos no kit
</commit_message>
<xml_diff>
--- a/apps/web/public/modelo_orcamento.xlsx
+++ b/apps/web/public/modelo_orcamento.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,6 +455,21 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>valor_unitario</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Fabricante</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
         </is>
       </c>
     </row>

</xml_diff>